<commit_message>
New Dashboard visuals and Power Query scripts
PBIP files has been updated with more dashboard visuals and Power Query scripts has been updated to use parameters for easier changes to files to be used.
</commit_message>
<xml_diff>
--- a/DataSource/Transaction Category.xlsx
+++ b/DataSource/Transaction Category.xlsx
@@ -1,42 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e088fed3854c41cd/Desktop/Anasabaziz Business/PowerBI Projects/Personal Finance Dashboard/DataSource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="285" documentId="8_{D883DFB9-DF3E-46C6-80F8-579E9D88C6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5836951E-AD00-45A3-AB06-672A6B012F71}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_3C7A3245A29E33DA2148BAA30415A3C0CDECE880" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{901F5F5A-B39C-41C8-AA0F-108C043226FE}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{4EDCB8B7-4CD2-4D62-A78A-444A93E1942A}"/>
+    <workbookView xWindow="7200" yWindow="1785" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Category" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="159">
+  <si>
+    <t>Financial Type</t>
+  </si>
   <si>
     <t>Category</t>
   </si>
@@ -47,402 +34,417 @@
     <t>Allocation Type</t>
   </si>
   <si>
-    <t>Financial Type</t>
+    <t>Expense</t>
+  </si>
+  <si>
+    <t>Automative</t>
+  </si>
+  <si>
+    <t>Automobile rental</t>
+  </si>
+  <si>
+    <t>Needs</t>
+  </si>
+  <si>
+    <t>Auto maintenance</t>
+  </si>
+  <si>
+    <t>Car wash</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Education - others</t>
+  </si>
+  <si>
+    <t>Elementary School</t>
+  </si>
+  <si>
+    <t>College &amp; University</t>
+  </si>
+  <si>
+    <t>Business School</t>
+  </si>
+  <si>
+    <t>Vocational School</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Household appliances</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Digital applications</t>
+  </si>
+  <si>
+    <t>Wants</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Photography store</t>
+  </si>
+  <si>
+    <t>Music</t>
+  </si>
+  <si>
+    <t>Gaming</t>
+  </si>
+  <si>
+    <t>Toys</t>
+  </si>
+  <si>
+    <t>Art &amp; craft store</t>
+  </si>
+  <si>
+    <t>Art gallery</t>
+  </si>
+  <si>
+    <t>Motion picture</t>
+  </si>
+  <si>
+    <t>Tourist Attractions</t>
+  </si>
+  <si>
+    <t>Amusement parks</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Money Transfer</t>
+  </si>
+  <si>
+    <t>Financial services</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Foreign currency</t>
+  </si>
+  <si>
+    <t>Investment</t>
+  </si>
+  <si>
+    <t>Investments</t>
+  </si>
+  <si>
+    <t>Taxes</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>Finances</t>
+  </si>
+  <si>
+    <t>Cash withdrawal</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>Food &amp; Beverage</t>
+  </si>
+  <si>
+    <t>Beverage</t>
+  </si>
+  <si>
+    <t>Grocery</t>
+  </si>
+  <si>
+    <t>Bakery</t>
+  </si>
+  <si>
+    <t>Food deliveries</t>
+  </si>
+  <si>
+    <t>Eating places &amp; restaurants</t>
+  </si>
+  <si>
+    <t>Caterers</t>
+  </si>
+  <si>
+    <t>Fast food restaurants</t>
+  </si>
+  <si>
+    <t>Health &amp; Beauty</t>
+  </si>
+  <si>
+    <t>Cosmetic stores</t>
+  </si>
+  <si>
+    <t>Hair saloon &amp; barber shops</t>
+  </si>
+  <si>
+    <t>Massage parlors</t>
+  </si>
+  <si>
+    <t>Health spas</t>
+  </si>
+  <si>
+    <t>Home &amp; Property</t>
+  </si>
+  <si>
+    <t>Pets</t>
+  </si>
+  <si>
+    <t>Garden supplies</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Furnishing</t>
+  </si>
+  <si>
+    <t>Real estate agents</t>
+  </si>
+  <si>
+    <t>Leisure &amp; Sports</t>
+  </si>
+  <si>
+    <t>Recreational camping</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Sporting goods</t>
+  </si>
+  <si>
+    <t>Sports club</t>
+  </si>
+  <si>
+    <t>Golf</t>
+  </si>
+  <si>
+    <t>Membership club</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Dental</t>
+  </si>
+  <si>
+    <t>Pharmacy</t>
+  </si>
+  <si>
+    <t>Optician</t>
+  </si>
+  <si>
+    <t>Medical services</t>
+  </si>
+  <si>
+    <t>Nursing care facilities</t>
+  </si>
+  <si>
+    <t>Other Expenses</t>
+  </si>
+  <si>
+    <t>Maritime</t>
+  </si>
+  <si>
+    <t>Religion</t>
+  </si>
+  <si>
+    <t>Tobacco</t>
+  </si>
+  <si>
+    <t>Charity &amp; social organisation</t>
+  </si>
+  <si>
+    <t>Organisation membership</t>
+  </si>
+  <si>
+    <t>Associations</t>
+  </si>
+  <si>
+    <t>Fines</t>
+  </si>
+  <si>
+    <t>Other expenses</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Property services</t>
+  </si>
+  <si>
+    <t>Printing services</t>
+  </si>
+  <si>
+    <t>Cleaning services</t>
+  </si>
+  <si>
+    <t>Freight &amp; courier services</t>
+  </si>
+  <si>
+    <t>Computer, network &amp; TV</t>
+  </si>
+  <si>
+    <t>Tailors &amp; alteration</t>
+  </si>
+  <si>
+    <t>Antique services</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Laundry services</t>
+  </si>
+  <si>
+    <t>Carpeting &amp; upholstery</t>
+  </si>
+  <si>
+    <t>Funeral services</t>
+  </si>
+  <si>
+    <t>Consulting services</t>
+  </si>
+  <si>
+    <t>Equipment rental</t>
+  </si>
+  <si>
+    <t>Legal services</t>
+  </si>
+  <si>
+    <t>Shopping</t>
+  </si>
+  <si>
+    <t>Jewellery &amp; watches</t>
+  </si>
+  <si>
+    <t>Stationery &amp; book store</t>
+  </si>
+  <si>
+    <t>Clothes</t>
+  </si>
+  <si>
+    <t>Shoes</t>
+  </si>
+  <si>
+    <t>Department stores</t>
+  </si>
+  <si>
+    <t>Sports &amp; shoes</t>
+  </si>
+  <si>
+    <t>Luggage &amp; leather goods</t>
+  </si>
+  <si>
+    <t>Sewing store</t>
+  </si>
+  <si>
+    <t>Telecommunications</t>
+  </si>
+  <si>
+    <t>Telecommunications - others</t>
+  </si>
+  <si>
+    <t>Mobile Equipment</t>
+  </si>
+  <si>
+    <t>Mobile Charges</t>
+  </si>
+  <si>
+    <t>Telegraphic Services</t>
+  </si>
+  <si>
+    <t>Transportation</t>
+  </si>
+  <si>
+    <t>Rail commute</t>
+  </si>
+  <si>
+    <t>Taxi &amp; limousines</t>
+  </si>
+  <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>Tolls</t>
+  </si>
+  <si>
+    <t>Petrol</t>
+  </si>
+  <si>
+    <t>Parking</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Airlines</t>
+  </si>
+  <si>
+    <t>Accomodation</t>
+  </si>
+  <si>
+    <t>Airport terminal</t>
+  </si>
+  <si>
+    <t>Travel Agency &amp; Tour</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Electric, water &amp; gas</t>
+  </si>
+  <si>
+    <t>Zakat</t>
+  </si>
+  <si>
+    <t>Zakat Pendapatan</t>
+  </si>
+  <si>
+    <t>Zakat Perniagaan</t>
+  </si>
+  <si>
+    <t>Zakat Simpanan</t>
+  </si>
+  <si>
+    <t>Zakat Pelaburan</t>
+  </si>
+  <si>
+    <t>Zakat KWSP</t>
+  </si>
+  <si>
+    <t>Zakat Emas</t>
+  </si>
+  <si>
+    <t>Zakat Perak</t>
+  </si>
+  <si>
+    <t>Qadha Zakat</t>
+  </si>
+  <si>
+    <t>Zakat Harta</t>
+  </si>
+  <si>
+    <t>Zakat Padi</t>
+  </si>
+  <si>
+    <t>Zakat Ternakan</t>
   </si>
   <si>
     <t>Income</t>
   </si>
   <si>
-    <t>Expense</t>
-  </si>
-  <si>
-    <t>Automative</t>
-  </si>
-  <si>
-    <t>Automobile rental</t>
-  </si>
-  <si>
-    <t>Auto maintenance</t>
-  </si>
-  <si>
-    <t>Car wash</t>
-  </si>
-  <si>
-    <t>Needs</t>
-  </si>
-  <si>
-    <t>Education</t>
-  </si>
-  <si>
-    <t>Education - others</t>
-  </si>
-  <si>
-    <t>Elementary School</t>
-  </si>
-  <si>
-    <t>Business School</t>
-  </si>
-  <si>
-    <t>Vocational School</t>
-  </si>
-  <si>
-    <t>Electronics</t>
-  </si>
-  <si>
-    <t>Household appliances</t>
-  </si>
-  <si>
-    <t>Computer</t>
-  </si>
-  <si>
-    <t>Digital applications</t>
-  </si>
-  <si>
-    <t>Entertainment</t>
-  </si>
-  <si>
-    <t>Photography store</t>
-  </si>
-  <si>
-    <t>Music</t>
-  </si>
-  <si>
-    <t>Gaming</t>
-  </si>
-  <si>
-    <t>Art &amp; craft store</t>
-  </si>
-  <si>
-    <t>Art gallery</t>
-  </si>
-  <si>
-    <t>Motion picture</t>
-  </si>
-  <si>
-    <t>Tourist Attractions</t>
-  </si>
-  <si>
-    <t>Amusement parks</t>
-  </si>
-  <si>
-    <t>Wants</t>
-  </si>
-  <si>
-    <t>Financial Services</t>
-  </si>
-  <si>
-    <t>Money Transfer</t>
-  </si>
-  <si>
-    <t>Financial services</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Foreign currency</t>
-  </si>
-  <si>
-    <t>Investment</t>
-  </si>
-  <si>
-    <t>Taxes</t>
-  </si>
-  <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>Finances</t>
-  </si>
-  <si>
-    <t>Cash withdrawal</t>
-  </si>
-  <si>
-    <t>Payment</t>
-  </si>
-  <si>
-    <t>Food &amp; Beverage</t>
-  </si>
-  <si>
-    <t>Beverage</t>
-  </si>
-  <si>
-    <t>Grocery</t>
-  </si>
-  <si>
-    <t>Bakery</t>
-  </si>
-  <si>
-    <t>Eating places &amp; restaurants</t>
-  </si>
-  <si>
-    <t>Caterers</t>
-  </si>
-  <si>
-    <t>Fast food restaurants</t>
-  </si>
-  <si>
-    <t>Health &amp; Beauty</t>
-  </si>
-  <si>
-    <t>Cosmetic stores</t>
-  </si>
-  <si>
-    <t>Hair saloon &amp; barber shops</t>
-  </si>
-  <si>
-    <t>Massage parlors</t>
-  </si>
-  <si>
-    <t>Health spas</t>
-  </si>
-  <si>
-    <t>Home &amp; Property</t>
-  </si>
-  <si>
-    <t>Pets</t>
-  </si>
-  <si>
-    <t>Garden supplies</t>
-  </si>
-  <si>
-    <t>Maintenance</t>
-  </si>
-  <si>
-    <t>Furnishing</t>
-  </si>
-  <si>
-    <t>Real estate agents</t>
-  </si>
-  <si>
-    <t>Leisure &amp; Sports</t>
-  </si>
-  <si>
-    <t>Recreational camping</t>
-  </si>
-  <si>
-    <t>Bicycle</t>
-  </si>
-  <si>
-    <t>Sporting goods</t>
-  </si>
-  <si>
-    <t>Sports club</t>
-  </si>
-  <si>
-    <t>Golf</t>
-  </si>
-  <si>
-    <t>Membership club</t>
-  </si>
-  <si>
-    <t>Medical</t>
-  </si>
-  <si>
-    <t>Dental</t>
-  </si>
-  <si>
-    <t>Pharmacy</t>
-  </si>
-  <si>
-    <t>Optician</t>
-  </si>
-  <si>
-    <t>Medical services</t>
-  </si>
-  <si>
-    <t>Nursing care facilities</t>
-  </si>
-  <si>
-    <t>Other Expenses</t>
-  </si>
-  <si>
-    <t>Maritime</t>
-  </si>
-  <si>
-    <t>Religion</t>
-  </si>
-  <si>
-    <t>Tobacco</t>
-  </si>
-  <si>
-    <t>Charity &amp; social organisation</t>
-  </si>
-  <si>
-    <t>Organisation membership</t>
-  </si>
-  <si>
-    <t>Associations</t>
-  </si>
-  <si>
-    <t>Fines</t>
-  </si>
-  <si>
-    <t>Other expenses</t>
-  </si>
-  <si>
-    <t>Services</t>
-  </si>
-  <si>
-    <t>Property services</t>
-  </si>
-  <si>
-    <t>Printing services</t>
-  </si>
-  <si>
-    <t>Cleaning services</t>
-  </si>
-  <si>
-    <t>Freight &amp; courier services</t>
-  </si>
-  <si>
-    <t>Computer, network &amp; TV</t>
-  </si>
-  <si>
-    <t>Tailors &amp; alteration</t>
-  </si>
-  <si>
-    <t>Antique services</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Laundry services</t>
-  </si>
-  <si>
-    <t>Carpeting &amp; upholstery</t>
-  </si>
-  <si>
-    <t>Funeral services</t>
-  </si>
-  <si>
-    <t>Consulting services</t>
-  </si>
-  <si>
-    <t>Equipment rental</t>
-  </si>
-  <si>
-    <t>Legal services</t>
-  </si>
-  <si>
-    <t>Shopping</t>
-  </si>
-  <si>
-    <t>Jewellery &amp; watches</t>
-  </si>
-  <si>
-    <t>Stationery &amp; book store</t>
-  </si>
-  <si>
-    <t>Clothes</t>
-  </si>
-  <si>
-    <t>Shoes</t>
-  </si>
-  <si>
-    <t>Department stores</t>
-  </si>
-  <si>
-    <t>Sports &amp; shoes</t>
-  </si>
-  <si>
-    <t>Luggage &amp; leather goods</t>
-  </si>
-  <si>
-    <t>Sewing store</t>
-  </si>
-  <si>
-    <t>Telecommunications</t>
-  </si>
-  <si>
-    <t>Telecommunications - others</t>
-  </si>
-  <si>
-    <t>Mobile Equipment</t>
-  </si>
-  <si>
-    <t>Mobile Charges</t>
-  </si>
-  <si>
-    <t>Telegraphic Services</t>
-  </si>
-  <si>
-    <t>Transportation</t>
-  </si>
-  <si>
-    <t>Rail commute</t>
-  </si>
-  <si>
-    <t>Taxi &amp; limousines</t>
-  </si>
-  <si>
-    <t>Petrol</t>
-  </si>
-  <si>
-    <t>Parking</t>
-  </si>
-  <si>
-    <t>Transport</t>
-  </si>
-  <si>
-    <t>Travel</t>
-  </si>
-  <si>
-    <t>Airlines</t>
-  </si>
-  <si>
-    <t>Accomodation</t>
-  </si>
-  <si>
-    <t>Airport terminal</t>
-  </si>
-  <si>
-    <t>Travel Agency &amp; Tour</t>
-  </si>
-  <si>
-    <t>Utilities</t>
-  </si>
-  <si>
-    <t>Electric, water &amp; gas</t>
-  </si>
-  <si>
-    <t>Zakat</t>
-  </si>
-  <si>
-    <t>Zakat Pendapatan</t>
-  </si>
-  <si>
-    <t>Zakat Perniagaan</t>
-  </si>
-  <si>
-    <t>Zakat Simpanan</t>
-  </si>
-  <si>
-    <t>Zakat Pelaburan</t>
-  </si>
-  <si>
-    <t>Zakat KWSP</t>
-  </si>
-  <si>
-    <t>Zakat Emas</t>
-  </si>
-  <si>
-    <t>Zakat Perak</t>
-  </si>
-  <si>
-    <t>Qadha Zakat</t>
-  </si>
-  <si>
-    <t>Zakat Harta</t>
-  </si>
-  <si>
-    <t>Zakat Padi</t>
-  </si>
-  <si>
-    <t>Zakat Ternakan</t>
-  </si>
-  <si>
     <t>Salary</t>
   </si>
   <si>
@@ -452,16 +454,7 @@
     <t>Crypto</t>
   </si>
   <si>
-    <t>Main</t>
-  </si>
-  <si>
-    <t>Secondary</t>
-  </si>
-  <si>
-    <t>College &amp; University</t>
-  </si>
-  <si>
-    <t>Toys</t>
+    <t>Asset</t>
   </si>
   <si>
     <t>Cash</t>
@@ -470,25 +463,40 @@
     <t>Credit Card Payment</t>
   </si>
   <si>
-    <t>Asset</t>
+    <t>Cash Transfer</t>
   </si>
   <si>
     <t>Transfer</t>
   </si>
   <si>
-    <t>Cash Transfer</t>
-  </si>
-  <si>
-    <t>Tolls</t>
-  </si>
-  <si>
-    <t>Bus</t>
-  </si>
-  <si>
-    <t>Investments</t>
-  </si>
-  <si>
-    <t>Food deliveries</t>
+    <t>Rent, Royalty, Premiums</t>
+  </si>
+  <si>
+    <t>Dividend, Interest, Discounts</t>
+  </si>
+  <si>
+    <t>Gains &amp; Profit from Employment</t>
+  </si>
+  <si>
+    <t>Claims</t>
+  </si>
+  <si>
+    <t>Discounts</t>
+  </si>
+  <si>
+    <t>Rental Income</t>
+  </si>
+  <si>
+    <t>Royalty</t>
+  </si>
+  <si>
+    <t>Interest Income</t>
+  </si>
+  <si>
+    <t>Premiums</t>
+  </si>
+  <si>
+    <t>Gains &amp; Profit from Business</t>
   </si>
 </sst>
 </file>
@@ -543,14 +551,18 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D7219355-0FF9-4115-A0B2-7E8271BFD662}" name="Table1" displayName="Table1" ref="A1:D134" totalsRowShown="0">
-  <autoFilter ref="A1:D134" xr:uid="{D7219355-0FF9-4115-A0B2-7E8271BFD662}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D140" totalsRowShown="0">
+  <autoFilter ref="A1:D140" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{34AC46E0-4DA8-4773-A0EF-D3EAD565FC03}" name="Financial Type"/>
-    <tableColumn id="2" xr3:uid="{880D115D-E5A0-43A7-928A-ED1018A8494C}" name="Category"/>
-    <tableColumn id="3" xr3:uid="{DBB6EC90-E58E-4391-AD23-B4D4FA980CBA}" name="SubCategory"/>
-    <tableColumn id="4" xr3:uid="{55991010-F5A6-4D5E-8F6F-60C5F92378DE}" name="Allocation Type"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Financial Type"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Category"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="SubCategory"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Allocation Type"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -872,173 +884,173 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7519005C-4CC1-4FA5-8D52-72FAC0180C76}">
-  <dimension ref="A1:D134"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D140"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -1047,12 +1059,12 @@
         <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -1061,12 +1073,12 @@
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -1075,12 +1087,12 @@
         <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1089,1673 +1101,1757 @@
         <v>16</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>141</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D21" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D25" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D27" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D28" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D29" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D30" t="s">
-        <v>149</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D31" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C32" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" t="s">
         <v>37</v>
-      </c>
-      <c r="D32" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C33" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D34" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C36" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D36" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D38" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
-        <v>150</v>
+        <v>47</v>
       </c>
       <c r="D39" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D40" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D42" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D43" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D44" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C45" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D45" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B46" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D46" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D47" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C48" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D48" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C49" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D49" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B50" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D50" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D51" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C52" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D52" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D53" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B54" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C54" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D54" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B55" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C55" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D55" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B56" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C56" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D56" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B57" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D57" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B58" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C58" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D58" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B59" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C59" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D59" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B60" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C60" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D60" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C61" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D61" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B62" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C62" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D62" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B63" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D63" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B64" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C64" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D64" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B65" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C65" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D65" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B66" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C66" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D66" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B67" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D67" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C68" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D68" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B69" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C69" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D69" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C70" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D70" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C71" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D71" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B72" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C72" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D72" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B73" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C73" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D73" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B74" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C74" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D74" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B75" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C75" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D75" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B76" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C76" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D76" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B77" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C77" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D77" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B78" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C78" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D78" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B79" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C79" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D79" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B80" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C80" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D80" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B81" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C81" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B82" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C82" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D82" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B83" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C83" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D83" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B84" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D84" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B85" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C85" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D85" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B86" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C86" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D86" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B87" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C87" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B88" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C88" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D88" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B89" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C89" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D89" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B90" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C90" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D90" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B91" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C91" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D91" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B92" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C92" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D92" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B93" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C93" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D93" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B94" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C94" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D94" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C95" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D95" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B96" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C96" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D96" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B97" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C97" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D97" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C98" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D98" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B99" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C99" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D99" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B100" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C100" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D100" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B101" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C101" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D101" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B102" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C102" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D102" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B103" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C103" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D103" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B104" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C104" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D104" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B105" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C105" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D105" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B106" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C106" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D106" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B107" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C107" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="D107" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B108" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C108" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="D108" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B109" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C109" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D109" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B110" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C110" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D110" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B111" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C111" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D111" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B112" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C112" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D112" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B113" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C113" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D113" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B114" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C114" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D114" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B115" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C115" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D115" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B116" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C116" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D116" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B117" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C117" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D117" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B118" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C118" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D118" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B119" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C119" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D119" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B120" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C120" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D120" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B121" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C121" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D121" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B122" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C122" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D122" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B123" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C123" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D123" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B124" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C124" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D124" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B125" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C125" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D125" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B126" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C126" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D126" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B127" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C127" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D127" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B128" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C128" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D128" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B129" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C129" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D129" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>4</v>
+        <v>140</v>
       </c>
       <c r="B130" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="C130" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D130" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>4</v>
+        <v>140</v>
       </c>
       <c r="B131" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="C131" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="D131" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>4</v>
+        <v>140</v>
       </c>
       <c r="B132" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="C132" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D132" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B133" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C133" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="D133" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
+        <v>140</v>
+      </c>
+      <c r="B134" t="s">
+        <v>150</v>
+      </c>
+      <c r="C134" t="s">
+        <v>153</v>
+      </c>
+      <c r="D134" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>140</v>
+      </c>
+      <c r="B135" t="s">
+        <v>149</v>
+      </c>
+      <c r="C135" t="s">
+        <v>154</v>
+      </c>
+      <c r="D135" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>140</v>
+      </c>
+      <c r="B136" t="s">
+        <v>149</v>
+      </c>
+      <c r="C136" t="s">
+        <v>155</v>
+      </c>
+      <c r="D136" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>140</v>
+      </c>
+      <c r="B137" t="s">
+        <v>149</v>
+      </c>
+      <c r="C137" t="s">
+        <v>157</v>
+      </c>
+      <c r="D137" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>140</v>
+      </c>
+      <c r="B138" t="s">
+        <v>158</v>
+      </c>
+      <c r="C138" t="s">
+        <v>143</v>
+      </c>
+      <c r="D138" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>144</v>
       </c>
-      <c r="B134" t="s">
-        <v>142</v>
-      </c>
-      <c r="C134" t="s">
+      <c r="B139" t="s">
+        <v>145</v>
+      </c>
+      <c r="C139" t="s">
         <v>146</v>
       </c>
-      <c r="D134" t="s">
+      <c r="D139" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>144</v>
+      </c>
+      <c r="B140" t="s">
         <v>145</v>
+      </c>
+      <c r="C140" t="s">
+        <v>147</v>
+      </c>
+      <c r="D140" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>